<commit_message>
feat: restructure design doc into IA 8 categories (28 screens)
- adopt user IA (8 top-level categories): dashboard/monitoring, allocation,
  model mgmt, marketplace, events/alerts, board, audit/security, system settings
- closed-network (public deployment) premise: in-app alerts (no mail),
  offline model import with security scan, audit trail (1yr+)
- 19 -> 28 screens; mark IA new/updated screens with badges
- sync routing/shell/screen-data/schema/checklist/roadmap + regenerate IA xlsx

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/for_claude/anclave-ia.xlsx
+++ b/for_claude/anclave-ia.xlsx
@@ -8,13 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="화면 IA" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="표시 데이터" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="승인 구조" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="승인 구조" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="전제·정책" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'화면 IA'!$A$1:$I$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'표시 데이터'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'승인 구조'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'화면 IA'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'승인 구조'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'전제·정책'!$A$1:$B$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -456,18 +456,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -478,7 +477,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>그룹</t>
+          <t>IA 대분류</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -498,20 +497,15 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>상위·진입</t>
+          <t>주요 액션·프로세스</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>주요 액션·프로세스</t>
+          <t>표시 데이터</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>표시 데이터</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
@@ -525,42 +519,37 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
+          <t>1.대시보드·관제</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>로그인</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>/login</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>공통</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>로그인</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>/login</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>공통</t>
-        </is>
-      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>진입점</t>
+          <t>3계정 선택 → 역할별 첫 화면</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>admin/manager/user 3계정 선택 → 역할별 첫 화면</t>
+          <t>3계정·공통 비번</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>3계정 안내, 공통 비번</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>하드코딩 시연</t>
+          <t>하드코딩</t>
         </is>
       </c>
     </row>
@@ -572,40 +561,39 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>1.대시보드·관제</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>마켓플레이스</t>
+          <t>전체 서버 모니터링</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>/marketplace</t>
+          <t>/resource-map</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>A 전용</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>사이드바</t>
+          <t>전체 헬스 → MIG 현황 → 이벤트 → 서버 타일 클릭</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>서비스 열람 → 'API 요청' → B 승인 / 검색·필터</t>
+          <t>좌:자원맵(서버 타일+GPU4 미니) / 우상:전체 MIG 슬라이스 현황(빗금=가용·전체↔서버별) / 우하:전체 서버 이벤트 로그</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>서비스 table(명·종류·API여부·모델), 최대 사용량 순위 Top N</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr"/>
+          <t>메인·Step1 · 크리티컬 알람=정중앙 경고 · H100 4개/서버</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -615,40 +603,39 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>1.대시보드·관제</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>서비스 상세</t>
+          <t>단일 서버 모니터링</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>/marketplace/:id</t>
+          <t>/resource-map/:serverId</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>A 전용</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>마켓 → 클릭</t>
+          <t>자원맵 슬라이스 → KPI 추이 → GPU 테이블·서비스 → GPU 클릭</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>상세 열람, 토큰 사용량 확인</t>
+          <t>좌:자원맵(서버 GPU 전체·슬라이스) / 우상:CPU·RAM·GPU KPI+꺾은선 / 우하:GPU 테이블+올라간 서비스(사용량순)</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>URL·테스트URL·모델·소개·매뉴얼, key별 사용량</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr"/>
+          <t>Step2 · 플로팅(이벤트=드로어) · ←뒤로</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -658,42 +645,37 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>1.대시보드·관제</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>모델 카탈로그</t>
+          <t>GPU 상세 모니터링</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>/models</t>
+          <t>/resource-map/:serverId/:gpuId</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>공통 열람</t>
+          <t>A 전용</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>사이드바</t>
+          <t>KPI 추이 → 슬라이스·활동 → 올라간 서비스 → 워크스페이스 통로</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>열람(인기·사용량) / (A)신규 등록 / 검색·필터</t>
+          <t>KPI 꺾은선 · 슬라이스 분할(사용자·모델·컨테이너) · 최근활동 · 올라간 서비스 상세</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>모델 table(명·종류·사용량·부가), 인기 순위</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>사용자 신청 없음 · 추가는 관리자만</t>
+          <t>Step3 · ①비교·②자원맵 제외 · 워크스페이스 진입 버튼</t>
         </is>
       </c>
     </row>
@@ -705,40 +687,39 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>1.대시보드·관제</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>모델 상세</t>
+          <t>내 할당 자원 (실무 대시보드)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>/models/:id</t>
+          <t>/dashboard</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>B=C</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>카탈로그 → 클릭</t>
+          <t>자기 할당 GPU 상태 → 사용량·로그 → 콘솔/주피터</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>메타·사용량 확인, GPU 신청 시 이 모델 선택</t>
+          <t>GPU 상태(작업률·VRAM·CPU·MEM·온도·전력) · 토큰 사용량 · 네트워크 · 로그</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>메타데이터, 사용량</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr"/>
+          <t>본인 화면 · 할당 없으면 자원 신청현황으로</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -748,40 +729,39 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>1.대시보드·관제</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>게시판·공지</t>
+          <t>자원 신청현황</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>/board</t>
+          <t>/requests/status</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>B=C</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>사이드바</t>
+          <t>승인 전 내 신청 목록 확인 → 반려 사유</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>(B=C)문의 작성 / (A)답변·공지</t>
+          <t>내 신청 목록(대기/승인/반려)</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>공지/문의 탭, 글, 답변됨 배지, 상세 모달</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr"/>
+          <t>호스팅 전 사용자 첫 진입</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -791,42 +771,37 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>1.대시보드·관제</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>알림</t>
+          <t>관제 모니터링</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>/notifications</t>
+          <t>/admin/monitoring</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>공통</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>헤더 벨</t>
+          <t>상시 관제 빅스크린</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>승인/반려/에러 알림 확인, 모두 읽음</t>
+          <t>실시간 종합 대시보드(헬스·부하·알럿)</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>벨 드롭다운, 알림 목록, 메일 발송</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>글로벌 알림창</t>
+          <t>관제실</t>
         </is>
       </c>
     </row>
@@ -838,44 +813,35 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>자원맵·모니터링</t>
+          <t>2.할당 관리</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>전체 서버 모니터링</t>
+          <t>신청 관리</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>/resource-map</t>
+          <t>/requests</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>A 전용</t>
+          <t>B=C</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>관리자 메인(첫 진입) · Step 1</t>
+          <t>탭[API / GPU·모델 번들(공문 첨부) / 게시] → 상태 추적</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>전체 헬스 스캔 → MIG 현황 → 이벤트 → 서버 타일 클릭 → 단일</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>좌: 자원맵(서버 타일+GPU 4개 미니, 헬스 히트맵) / 우상: 전체 MIG 슬라이스 현황(크기별 개수·점유·빗금=가용·전체↔서버별 토글) / 우하: 전체 서버 이벤트 로그(/events 요약)</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>★ 메인 · 크리티컬 알람 = 정중앙 센터 경고 · H100 4개/서버 다수</t>
-        </is>
-      </c>
+          <t>내 신청 목록·상태 배지·번들 신청서·결과</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -885,42 +851,37 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>자원맵·모니터링</t>
+          <t>2.할당 관리</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>단일 서버 모니터링</t>
+          <t>게시 승인 관리</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>/resource-map/:serverId</t>
+          <t>/admin/approvals/publish</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>A 전용</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>전체 → 서버 타일 클릭 · Step 2</t>
+          <t>게시 신청 검토 → 승인(노출)/반려 → 앱 내 알림</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>자원맵 슬라이스 파악 → KPI 추이 → GPU 테이블·서비스 → GPU 클릭 → GPU 상세</t>
+          <t>게시 신청 목록·검토 상세</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>좌: 자원맵(서버 GPU 전체·슬라이스 분할/할당) / 우상: CPU·RAM·GPU KPI+꺾은선 추이 / 우하: GPU 상세 시각화 테이블 + 올라간 서비스(사용량순)</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>Step 2 · 플로팅(콘솔·주피터·이벤트 드로어) · ← Step 뒤로</t>
+          <t>독립 페이지</t>
         </is>
       </c>
     </row>
@@ -932,42 +893,37 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>자원맵·모니터링</t>
+          <t>2.할당 관리</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>GPU 상세 모니터링</t>
+          <t>GPU 승인 관리</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>/resource-map/:serverId/:gpuId</t>
+          <t>/admin/approvals/gpu</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>A 전용</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>단일 서버 → GPU 클릭 · Step 3</t>
+          <t>스펙·사유·공문 확인 → 승인(자원맵 서버 선택)/반려</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>KPI 추이 → 슬라이스·활동 → 올라간 서비스 → 워크스페이스 통로</t>
+          <t>탭[승인 대기 / 기 승인·반려] · 자원맵 서버 선택</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>KPI 꺾은선(작업률·VRAM·온도·전력) · 슬라이스 분할(사용자·모델·컨테이너) · 최근활동 타임라인 · 올라간 서비스 상세</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>Step 3 · ①비교·②자원맵 제외 · 워크스페이스 진입 버튼 · 플로팅 · ← Step 뒤로</t>
+          <t>독립 · 변경/회수 승인도</t>
         </is>
       </c>
     </row>
@@ -979,40 +935,39 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>신청·승인</t>
+          <t>2.할당 관리</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>신청 관리</t>
+          <t>변경·확장·이전·회수</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>/requests</t>
+          <t>/requests/gpu-change</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>B=C</t>
+          <t>B=C 신청 / A 승인</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>사이드바</t>
+          <t>신청 → 4케이스(expand/migrate/change/reclaim) · 관리자 직접 회수(유휴 탐지)</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>3탭(API/GPU 마법사/게시) 신청 → 상태 추적 → 결과</t>
+          <t>변경 신청 · 케이스별 결과 · 자원맵 전/후</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>신청 목록, 상태 배지(승인/대기/반려), GPU 마법사, 결과(key·할당·사유)</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr"/>
+          <t>회수 권고 알림</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1022,42 +977,37 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>신청·승인</t>
+          <t>3.모델 관리</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>게시 승인 관리</t>
+          <t>모델 카탈로그</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>/admin/approvals/publish</t>
+          <t>/models</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>공통 열람</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>사이드바</t>
+          <t>열람(인기·사용량) / (A)신규 반입·버전 관리</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>게시 신청 상세 검토 → 승인(마켓 노출)/반려(사유) → 알림</t>
+          <t>모델 목록(버전)·인기 순위</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>게시 신청 목록, 검토 상세</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>독립 페이지</t>
+          <t>사용자 신청 없음·도입은 게시판</t>
         </is>
       </c>
     </row>
@@ -1069,44 +1019,35 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>신청·승인</t>
+          <t>3.모델 관리</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>GPU 승인 관리</t>
+          <t>모델 상세</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>/admin/approvals/gpu</t>
+          <t>/models/:id</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>사이드바</t>
+          <t>메타·사용량 / GPU 신청 시 선택</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>GPU 신청 사유·스펙·모델 검토 → 승인(자원맵 서버 선택)/반려</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>GPU 신청(사유·스펙·요청 모델), 자원맵 서버 선택, 반려 사유 모달</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>독립 페이지 · GPU 추가/변경/회수 승인도 여기</t>
-        </is>
-      </c>
+          <t>메타데이터(권장 GPU·라이선스)·사용량</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1116,42 +1057,37 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>신청·승인</t>
+          <t>3.모델 관리</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>실무관리자 대시보드 = 사용자 자원 모니터링</t>
+          <t>신규 모델 반입</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>/dashboard</t>
+          <t>/admin/models/new</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>B=C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>호스팅 보유자 첫 진입</t>
+          <t>격리 업로드 → 보안 점검 → 메타데이터 → 버전</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>자기 할당 GPU 상태 확인 → 사용량·로그 → 콘솔/주피터 접속</t>
+          <t>보안 점검(safetensors 강제·modelscan·picklescan·체크섬·서명)·진행률</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>GPU 상태(작업률·VRAM·CPU·MEM·온도·전력), 토큰 사용량, 네트워크, 로그, 콘솔/주피터</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>사용자 본인 화면 · 드릴다운 아님</t>
+          <t>폐쇄망 오프라인 반입·보안관문</t>
         </is>
       </c>
     </row>
@@ -1163,44 +1099,35 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>신청·승인</t>
+          <t>3.모델 관리</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>GPU 추가/변경/회수</t>
+          <t>내 모델</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>/requests/gpu-change</t>
+          <t>/models/mine</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>B=C 신청 / A 승인</t>
+          <t>B=C</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>신청관리·대시보드</t>
+          <t>내가 쓰는 모델 목록 · 도입은 게시판 문의</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>변경 사유·스펙 → A 승인 4케이스(expand/migrate/change/reclaim)</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>변경 신청 내역, 케이스별 더미 결과, 자원맵 반영 전/후</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>더미 UI · 승인은 GPU 승인 관리에서</t>
-        </is>
-      </c>
+          <t>내 모델 목록</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1210,42 +1137,37 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>신청·승인</t>
+          <t>3.모델 관리</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>받은 API 신청 승인</t>
+          <t>데몬·에이전트 관리</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>/api-approvals</t>
+          <t>/admin/agents</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>사이드바</t>
+          <t>노드 합류 시 자동 배포 · 상태/버전</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>받은 API 신청 검토 → 승인(key 발급/복사)/반려(사유) → 알림</t>
+          <t>노드별 에이전트(상태·버전)</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>받은 API 신청 목록, key별 호출량·연결 사용률 그래프</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>소유자 권한</t>
+          <t>최소권한·감사</t>
         </is>
       </c>
     </row>
@@ -1257,40 +1179,35 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>A 전용</t>
+          <t>4.마켓플레이스</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>신규 모델 도입</t>
+          <t>마켓플레이스</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>/admin/models/new</t>
+          <t>/marketplace</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>모델 카탈로그 '신규 등록'</t>
+          <t>AI 목록 탐색·검색·태그 → API 요청</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>업로드 → 보안 스캐닝 → 메타데이터 → 세팅 → 등록 완료</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>스캐닝 진행률, 메타데이터 폼</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr"/>
+          <t>서비스(명/종류/API/모델)·최대 사용량 순위</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1300,44 +1217,35 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>A 전용</t>
+          <t>4.마켓플레이스</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>에러·이벤트 관제</t>
+          <t>서비스(AI) 상세</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>/events</t>
+          <t>/marketplace/:id</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>A / B</t>
+          <t>공통</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>알럿 발생 / 사이드바</t>
+          <t>상세 열람 · 플레이그라운드 체험</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>알럿 → 이벤트 목록(심각도) → 상세 드로어 → 문제 GPU</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>이벤트 타임라인(위험/경고/정보/복구), 상세 드로어(상태·담당·조치), 검색·필터</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>알럿 시 메일 수신</t>
-        </is>
-      </c>
+          <t>URL·모델·매뉴얼·key별 사용량 · 플레이그라운드</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1347,94 +1255,450 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>A 전용</t>
+          <t>4.마켓플레이스</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>관제 모니터링</t>
+          <t>API 연동 (받은 API 승인)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>/admin/monitoring</t>
+          <t>/api-approvals</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>사이드바</t>
+          <t>받은 API 검토 → 승인(key 발급)/반려</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>상시 관제(빅스크린)</t>
+          <t>받은 API 목록 · key별 호출량 · 사용 가이드</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>실시간 빅스크린 대시보드, 개인정보 접근·관리자 활동 로그</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>관제실</t>
+          <t>쿼터·레이트리밋 추후</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>4.20</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>4.마켓플레이스</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>활성화 대시보드</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>/marketplace/activation</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>공통</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>발행자/소비자/관리자 뷰</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>발행자(내 토큰)·소비자(내 호출)·관리자(전체 귀속=모델×소비자×시간)</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>4.21</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>5.이벤트·알림</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>에러·이벤트 관제</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>/events</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>A / B</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>알럿 → 이벤트 목록 → 상세 드로어 → 문제 GPU</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>이벤트 타임라인(위험/경고/정보/복구)·XID/HW 에러·상세 드로어</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>앱 내 알림</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>4.22</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>5.이벤트·알림</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>알림 센터</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>/notifications</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>공통</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>알림 확인·모두 읽음</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>벨·알림 목록·3종(할당·승인/헬스·에러/회수 권고)</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>앱 내(메일 미사용)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>4.23</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>6.게시판</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>게시판·공지</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>/board</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>공통</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>(B=C)문의(모델 도입 요청) / (A)답변·공지</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>공지/문의·Q&amp;A/소개·매뉴얼 탭</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>4.24</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>7.감사·보안</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>감사 로그</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>/admin/audit</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>행위 추적 검색·필터</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>콘솔 접속·API 호출(소비자별)·권한/할당 변경 기록</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>1년+ 보관(공공 납품 요건)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>4.25</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>7.감사·보안</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>접근통제·권한</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>/admin/access</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>권한 정책 관리</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>권한 정책 목록</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>관리자/사용자 분리</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>4.26</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>8.시스템 설정</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>능력 탐지·기능 플래그</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>/admin/settings/capabilities</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>GPU·MIG 탐지 · 기능 on/off</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>지원 매트릭스(GPU·오케스트레이터)</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>노드 합류 시 재탐지·확정 필요</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>4.27</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>8.시스템 설정</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>사용자·역할 관리</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>/admin/settings/users</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>역할 관리·알림 채널 설정</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>사용자 목록(최종/실무/사용)</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>폐쇄망 내부 전달</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>4.28</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>8.시스템 설정</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>인프라 연동</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>/admin/settings/infra</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>모니터링·오케스트레이터 연동</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>DCGM·Prometheus·추론서버 /metrics·오케스트레이터</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>개념(페이지 아님)</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>워크스페이스</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>B=C / A</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>대시보드·GPU 상세 내 버튼</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>콘솔/주피터 버튼으로 접속</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>콘솔/주피터 버튼 접속</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>(데모 연결 미정)</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>추상 개념 · GPU 상세에 진입 통로</t>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>GPU 상세·대시보드 내 통로</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1"/>
+  <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1445,590 +1709,206 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>그룹</t>
+          <t>승인 종류</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>화면</t>
+          <t>신청자</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>핵심 지표(크게)</t>
+          <t>승인 주체</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>목록/테이블</t>
+          <t>처리 페이지</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>차트·시각화</t>
+          <t>승인 결과</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>상태·액션</t>
+          <t>반려·통보</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>자원맵·모니터링</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>게시 승인</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>전체 서버 모니터링 (메인·Step1·A)</t>
+          <t>B/C · A 직접</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>전체 GPU 가동률·서버 수·장애 대수</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>우상: 전체 MIG 슬라이스 현황(크기별 개수·점유·빗금=가용·전체↔서버별)</t>
+          <t>게시 승인 관리(4.9)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>좌: 자원맵 헬스 히트맵 / 우하: 전체 서버 이벤트 로그</t>
+          <t>마켓 노출</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>헬스 🟢🔴⚪ · 크리티컬 알람=정중앙 센터 경고 · 서버 타일→단일</t>
+          <t>반려 사유 · 앱 내 알림</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>자원맵·모니터링</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>GPU 신청 승인 (모델·공문 포함)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>단일 서버 모니터링 (Step2·A)</t>
+          <t>B/C</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>우상: CPU·RAM·GPU 값</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>우하: GPU 상세 테이블 · 올라간 서비스(사용량순)</t>
+          <t>GPU 승인 관리(4.10)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>좌: 자원맵(서버 GPU 전체·슬라이스) · 우상 KPI 꺾은선</t>
+          <t>자원맵 서버 선택 → 슬라이스 배치</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>GPU 클릭→GPU 상세 · 플로팅(이벤트=드로어) · ← Step 뒤로</t>
+          <t>반려 사유 · 앱 내 알림</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>자원맵·모니터링</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>변경·확장·이전·회수 승인</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>GPU 상세 모니터링 (Step3·A)</t>
+          <t>B/C</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>작업률·VRAM·온도·전력 (꺾은선)</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>슬라이스 분할(사용자·모델·컨테이너) · 올라간 서비스 상세</t>
+          <t>GPU 승인 관리(4.10)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>KPI 꺾은선(프로그레스바 제외) · 최근활동 타임라인</t>
+          <t>expand/migrate/change/reclaim</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>워크스페이스 통로 · 플로팅 · ← Step 뒤로 (①비교·②자원맵 제외)</t>
+          <t>반려 사유 · 회수 권고 알림</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>자원맵·모니터링</t>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>API 사용 승인 (외부 연동)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>사용자 자원 모니터링 (=대시보드·B=C)</t>
+          <t>타 사용자</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>내 GPU 작업률·VRAM·CPU·MEM·온도·전력</t>
+          <t>B(소유자)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>로그 · 나의 서비스 목록</t>
+          <t>API 연동(4.19)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>토큰 사용량 라인 · 네트워크</t>
+          <t>API key 수동 발급</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>콘솔 ▶/주피터 ▶ · 본인 화면(드릴다운 아님)</t>
+          <t>반려 사유 · 앱 내 알림</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>마켓·모델</t>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>모델 도입</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>마켓플레이스</t>
+          <t>B/C (요청)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>최대 사용량 서비스 순위</t>
+          <t>A (반입)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>서비스 — 명/종류/API여부/모델</t>
+          <t>게시판 문의 → 신규 모델 반입(4.14)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>사용량 Top N 바</t>
+          <t>보안 점검 후 카탈로그 노출</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>'API 요청' 버튼 · 검색·필터</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>마켓·모델</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>서비스 상세</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>토큰 사용량 합계</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>key(토큰)별 사용량</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>토큰 사용 추이 라인</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>URL·테스트URL·모델·소개·매뉴얼</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>마켓·모델</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>모델 카탈로그</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>인기·사용량 순위</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>모델 — 명/종류/사용량/부가서비스</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>사용량 바</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>(A)'신규 모델 등록' · 사용자 신청 없음</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>마켓·모델</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>모델 상세</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>사용량</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>메타데이터</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>사용 추이</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>GPU 신청 시 이 모델 선택</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>신청·승인·운영</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>신청 관리(B=C)</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>신청별 처리 상태</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>3탭(API/GPU/게시) 신청 목록</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
           <t>—</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>승인🟢/대기🟡/반려🔴·결과(key·할당·사유)·마법사</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>신청·승인·운영</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>게시 승인 관리(A)</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>대기 건수</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>게시 신청 목록</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>승인(마켓 노출) / 반려 사유 모달</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>신청·승인·운영</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>GPU 승인 관리(A)</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>대기 건수</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>GPU 신청 — 사유·스펙·요청 모델</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>승인→자원맵 서버 선택 · 반려 사유 모달</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>신청·승인·운영</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>GPU 추가/변경/회수</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>변경 신청 내역</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>expand/migrate/change/reclaim · 자원맵 전/후</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>신청·승인·운영</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>받은 API 승인(B)</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>key별 호출량</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>받은 API 신청 목록</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>호출량 라인</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>승인/반려·API key 수동 발급·복사</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>신청·승인·운영</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>신규 모델 도입(A)</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>보안 스캐닝 진행률</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>업로드·스캔 진행</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>업로드→스캐닝→메타→세팅 위저드</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>신청·승인·운영</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>에러·이벤트 관제</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>미확인 알럿 수</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>이벤트 타임라인</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>심각도 점(위험/경고/정보/복구)</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>검색·필터 칩·상세 드로어·문제 GPU 링크</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>신청·승인·운영</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>관제 모니터링(A)</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>실시간 종합 지표</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>개인정보 접근·관리자 활동 로그</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>실시간 빅스크린 대시보드</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>상시 관제</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>신청·승인·운영</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>게시판·공지 / 알림</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>글·문의·답변 / 알림 목록</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>(A)공지·답변 (B=C)문의 · 벨 드롭다운·모두 읽음</t>
         </is>
       </c>
     </row>
@@ -2044,179 +1924,123 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>승인 종류</t>
+          <t>항목</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>신청자</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>승인 주체</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>처리 페이지</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>승인 결과</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>반려</t>
+          <t>내용</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>게시 승인 (마켓 등록)</t>
+          <t>타겟 환경</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>B/C · A 직접</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>게시 승인 관리(4.12)</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>마켓 노출</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>반려 사유</t>
+          <t>폐쇄망 공공 납품</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>GPU 신청 승인 (모델 선택 포함)</t>
+          <t>역할</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>B/C</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>GPU 승인 관리(4.13)</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>자원맵 서버 선택 → 자동 할당</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>반려 사유</t>
+          <t>A 최종관리자 / B=C 실무=사용 (권한 동일·호스팅 유무로 화면만)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>GPU 추가/변경/회수 승인</t>
+          <t>알림</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>B/C</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>GPU 승인 관리(4.13)</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>expand/migrate/change/reclaim 재할당</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>반려 사유</t>
+          <t>앱 내 알림만 (메일 미사용) · 3종: 할당·승인 / 헬스·에러 / 회수 권고</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>API 사용 승인 (외부 연동)</t>
+          <t>모델 반입</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>타 사용자</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>B(소유자)</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>받은 API 신청 승인(4.16)</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>API key 수동 발급</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>반려 사유</t>
+          <t>폐쇄망 오프라인 반입 · 보안 점검(safetensors 강제·modelscan·picklescan·체크섬·서명) · 관리자만</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>사용자 모델 도입</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>독립 신청 없음 → 게시판 문의로 관리자에 요청</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>감사·보안</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>콘솔 접속·API 호출·권한 변경 기록 · 접속기록 1년+ 보관(공공 요건)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>보류</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>API 쿼터·레이트리밋(추후) · 벤치마킹(제외)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>모니터링 드릴다운</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>전체→단일→GPU 상세 (A 전용) · 사용자 단위 종합 조회 화면 없음</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1"/>
+  <autoFilter ref="A1:B1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>